<commit_message>
fix: complete battery-swap and firmware regression work
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Overall_Validation.xlsx
+++ b/Documentation/Overall_Validation.xlsx
@@ -845,10 +845,10 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>8</v>
@@ -857,7 +857,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v1.107: doc audit - fix user manual vs code, refresh all stale documents
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Overall_Validation.xlsx
+++ b/Documentation/Overall_Validation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -795,16 +795,16 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H4" s="8" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>CO-025</t>
+          <t>CO-008</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>CO-026</t>
+          <t>CO-013</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>CO-027</t>
+          <t>CO-025</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -1723,17 +1723,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>CH-042</t>
+          <t>CO-026</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>شارژر (Charger)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>شروع شارژ با وصل ورودی</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1748,17 +1748,17 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>CH-004</t>
+          <t>CO-027</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>شارژر (Charger)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>تنظیم BULK</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1773,17 +1773,17 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CH-005</t>
+          <t>CO-028</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>شارژر (Charger)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>ABSORB</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1798,17 +1798,17 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>EL-001</t>
+          <t>CO-029</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>ارتباط با پنل (EspLink)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>CH_PD و بوت</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1823,17 +1823,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>EL-002</t>
+          <t>CO-030</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>ارتباط با پنل (EspLink)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>تله‌متری زنده</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1848,17 +1848,17 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>FL-001</t>
+          <t>CO-033</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>تشخیص خطا (Fault)</t>
+          <t>قطع‌ووصل خروجی (Changeover)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>قاعدهٔ پمپ</t>
+          <t>عملکرد واقعی خروجی</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1873,17 +1873,17 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>FL-002</t>
+          <t>CH-042</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>تشخیص خطا (Fault)</t>
+          <t>شارژر (Charger)</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>قاعدهٔ غیبت</t>
+          <t>شروع شارژ با وصل ورودی</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1898,17 +1898,17 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>FL-001</t>
+          <t>CH-004</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>شارژر (Charger)</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>راه‌اندازی</t>
+          <t>تنظیم BULK</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1923,17 +1923,17 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>FL-002</t>
+          <t>CH-005</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>شارژر (Charger)</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>قفل</t>
+          <t>ABSORB</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>FL-003</t>
+          <t>EL-001</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>ارتباط با پنل (EspLink)</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>قفل</t>
+          <t>CH_PD و بوت</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>FL-004</t>
+          <t>EL-002</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>ارتباط با پنل (EspLink)</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>کار عادی</t>
+          <t>تله‌متری زنده</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -1998,17 +1998,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>MP-021</t>
+          <t>FL-001</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>تشخیص خطا (Fault)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>قاعدهٔ پمپ</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -2023,17 +2023,17 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>MP-022</t>
+          <t>FL-002</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>تشخیص خطا (Fault)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>قاعدهٔ غیبت</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -2048,17 +2048,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>MP-025</t>
+          <t>FL-001</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>راه‌اندازی</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -2073,17 +2073,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>MP-023</t>
+          <t>FL-002</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>قفل</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -2098,17 +2098,17 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>MS-001</t>
+          <t>FL-003</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>اندازه‌گیری (Measurement)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Init</t>
+          <t>قفل</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>PR-001</t>
+          <t>FL-004</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>حفاظت (Protection)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>ماژول خاموش</t>
+          <t>کار عادی</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -2148,17 +2148,17 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>RT-006</t>
+          <t>MP-021</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>سیستم‌عامل و تسک‌ها (Rtos)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>watchdog poll و check-in</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2173,17 +2173,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>UI-036</t>
+          <t>MP-022</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>رفتار کلی چراغ سبز</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -2198,17 +2198,17 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>UI-005</t>
+          <t>MP-025</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>باتری خالیِ کامل (درصد صفر)</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2223,17 +2223,17 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>UI-015</t>
+          <t>MP-023</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Full 100/95 enter</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>UI-032</t>
+          <t>MS-001</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>اندازه‌گیری (Measurement)</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>خطای ۶: قطع باتری حین شارژ</t>
+          <t>Init</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2273,20 +2273,170 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
+          <t>PR-001</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>حفاظت (Protection)</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>ماژول خاموش</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>RT-006</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>سیستم‌عامل و تسک‌ها (Rtos)</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>watchdog poll و check-in</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>UI-036</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>رفتار کلی چراغ سبز</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>UI-005</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>باتری خالیِ کامل (درصد صفر)</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>UI-015</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Full 100/95 enter</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>UI-032</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>خطای ۶: قطع باتری حین شارژ</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
           <t>UI-033</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>چراغ و بوق (UI)</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>خطای ۷: خرابی یک کانال شارژ</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>باز کردن فایل</t>
         </is>
@@ -2324,6 +2474,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Unify input Schmitt permission and harden ESP calibration clock
Share q33/q34 input limits with panel-adjustable q169/q170 re-arm margins across charger, MCU power path, UI presence, and Fault case-2. Preserve charger settle, MCU qualification, PB4 reconnect, and separate OV limits. Fix ESP_Calibration clock persistence/boot ordering with paired clock/board anchors, legacy stamp preservation, and bounded boot grace. Update panels, previews, simulators, docs, workbooks, and host tests.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Overall_Validation.xlsx
+++ b/Documentation/Overall_Validation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -848,7 +848,7 @@
         <v>17</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>8</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>1</v>
@@ -954,10 +954,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>2</v>
@@ -1004,10 +1004,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1998,17 +1998,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>FL-001</t>
+          <t>EL-030</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>تشخیص خطا (Fault)</t>
+          <t>ارتباط با پنل (EspLink)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>قاعدهٔ پمپ</t>
+          <t>ماندگاری حاشیه‌های اشمیت ورودی</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>FL-002</t>
+          <t>FL-001</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>قاعدهٔ غیبت</t>
+          <t>قاعدهٔ پمپ</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -2048,17 +2048,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>FL-001</t>
+          <t>FL-002</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>تشخیص خطا (Fault)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>راه‌اندازی</t>
+          <t>قاعدهٔ غیبت</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -2073,17 +2073,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>FL-002</t>
+          <t>FL-011</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>قفل خواندن حافظه (FlashLock)</t>
+          <t>تشخیص خطا (Fault)</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>قفل</t>
+          <t>اشمیت مشترک ورودی</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>FL-003</t>
+          <t>FL-001</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>قفل</t>
+          <t>راه‌اندازی</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>FL-004</t>
+          <t>FL-002</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>کار عادی</t>
+          <t>قفل</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -2148,17 +2148,17 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>MP-021</t>
+          <t>FL-003</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>قفل</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2173,17 +2173,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>MP-022</t>
+          <t>FL-004</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>تغذیهٔ میکرو (McuPowerPath)</t>
+          <t>قفل خواندن حافظه (FlashLock)</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>عملکرد واقعی مسیر تغذیه</t>
+          <t>کار عادی</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>MP-025</t>
+          <t>MP-021</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>MP-023</t>
+          <t>MP-022</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>MS-001</t>
+          <t>MP-025</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>اندازه‌گیری (Measurement)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Init</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>PR-001</t>
+          <t>MP-023</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>حفاظت (Protection)</t>
+          <t>تغذیهٔ میکرو (McuPowerPath)</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>ماژول خاموش</t>
+          <t>عملکرد واقعی مسیر تغذیه</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2298,17 +2298,17 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>RT-006</t>
+          <t>MS-001</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>سیستم‌عامل و تسک‌ها (Rtos)</t>
+          <t>اندازه‌گیری (Measurement)</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>watchdog poll و check-in</t>
+          <t>Init</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2323,17 +2323,17 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>UI-036</t>
+          <t>PR-001</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>حفاظت (Protection)</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>رفتار کلی چراغ سبز</t>
+          <t>ماژول خاموش</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>UI-005</t>
+          <t>RT-006</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>چراغ و بوق (UI)</t>
+          <t>سیستم‌عامل و تسک‌ها (Rtos)</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>باتری خالیِ کامل (درصد صفر)</t>
+          <t>watchdog poll و check-in</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>UI-015</t>
+          <t>UI-036</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Full 100/95 enter</t>
+          <t>رفتار کلی چراغ سبز</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>UI-032</t>
+          <t>UI-005</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>خطای ۶: قطع باتری حین شارژ</t>
+          <t>باتری خالیِ کامل (درصد صفر)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -2423,20 +2423,70 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
+          <t>UI-015</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Full 100/95 enter</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>UI-032</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>چراغ و بوق (UI)</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>خطای ۶: قطع باتری حین شارژ</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>باز کردن فایل</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
           <t>UI-033</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>چراغ و بوق (UI)</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>خطای ۷: خرابی یک کانال شارژ</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>باز کردن فایل</t>
         </is>
@@ -2480,6 +2530,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: audit STM32 + refresh all docs; remove charge CSV duration column (v1.117)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Overall_Validation.xlsx
+++ b/Documentation/Overall_Validation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="نمای کلی" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مرحله اول" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>